<commit_message>
Servicio detallado de exportacion funcionando
</commit_message>
<xml_diff>
--- a/InformeFinal.XLSX
+++ b/InformeFinal.XLSX
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>INFORME DE TAREAS POR CADA UNA DE LA ACTIVIDADES DEL CONTRATO DE PRESTACIÓN DE SERVICIOS</t>
   </si>
@@ -55,24 +55,6 @@
   </si>
   <si>
     <t>CANTIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brindar apoyo y acompañamiento técnico a los diferentes servidores públicos, contratistas y dependencias, en temas relacionados con tecnología para que éstos puedan adelantar en debida manera sus labores y cumplir así con los objetivos del plan de desarrollo. </t>
-  </si>
-  <si>
-    <t>Coadyuvar con las actividades del proceso del Sistema de Gestión de Calidad.</t>
-  </si>
-  <si>
-    <t>Las demás que correspondan y sean inherentes al objeto del contrato y le sean asignadas por el supervisor de la ejecución del contrato.</t>
-  </si>
-  <si>
-    <t>Realizar apoyo técnico en la intervención y correcto funcionamiento de la red.</t>
-  </si>
-  <si>
-    <t>Verificar el correcto funcionamiento del hardware y software de los equipos de la Administración Municipal con el propósito de que los trámites a realizar se efectúen con más eficiencia en beneficio de la comunidad en general.</t>
-  </si>
-  <si>
-    <t>TOTAL ACTIVIDADES</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha de informe:  </t>
@@ -100,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,14 +98,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -216,8 +190,65 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -227,72 +258,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,337 +565,229 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="20"/>
+      <c r="C3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6">
+      <c r="B5" s="18"/>
+      <c r="C5" s="19">
         <v>1040040179</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+    </row>
+    <row r="7" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="8" t="s">
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-    </row>
-    <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="I7" s="24"/>
+      <c r="J7" s="25"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="31"/>
+    </row>
+    <row r="9" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="9">
-        <v>185</v>
-      </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="B9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="9">
-        <v>60</v>
-      </c>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="9">
-        <v>48</v>
-      </c>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="B10" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" ht="39" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="9">
-        <v>39</v>
-      </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="B11" s="12"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="9">
-        <v>88</v>
-      </c>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="B12" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="9">
-        <f>SUM(F8:G12)</f>
-        <v>420</v>
-      </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-    </row>
-    <row r="15" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+    </row>
+    <row r="13" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-    </row>
-    <row r="16" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-    </row>
-    <row r="17" spans="1:10" ht="39" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-    </row>
-    <row r="19" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="F8:J8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="F9:J9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="F7:J7"/>
+  <mergeCells count="20">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="H8:J8"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:J2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:J3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:F12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>